<commit_message>
data: 2026-07-16 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daily" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1005,6 +1005,37 @@
         <v>95.06999999999999</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>9866</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>9142873.720000001</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>7853418.78</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>1289454.94</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>4.8692</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>926.71</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>80.56999999999999</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>95.14</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-17 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1036,6 +1036,37 @@
         <v>95.14</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>9872</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>9134811.77</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>7853426.25</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>1281385.52</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>4.8661</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>925.33</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>95.16</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-18 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1067,6 +1067,37 @@
         <v>95.16</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>9871</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>9144251.82</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>7852340.49</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>1291911.33</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>4.8763</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>926.38</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>80.56</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>95.14</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-19 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,37 @@
         <v>95.14</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>9878</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>9152459.810000001</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>7856829.4</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>1295630.4</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>4.8692</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>926.55</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>80.53</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>95.13</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-20 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1129,6 +1129,37 @@
         <v>95.13</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>9870</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>9145431.24</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>7856913.84</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>1288517.4</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>4.8338</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>926.59</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>95.18000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-21 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1160,6 +1160,37 @@
         <v>95.18000000000001</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>9871</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>9142716.560000001</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>7849287.57</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>1293428.99</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>926.22</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>80.62</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>95.18000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-22 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1191,6 +1191,37 @@
         <v>95.18000000000001</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>9873</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>9141365.390000001</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>7849351.97</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>1292013.41</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>925.9</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>80.63</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>95.19</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-23 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,6 +1222,37 @@
         <v>95.19</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>9894</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>9684264.109999999</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>8360766.58</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>1323497.53</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>4.8221</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>978.8</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>81.31999999999999</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>95.41</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-24 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1253,6 +1253,37 @@
         <v>95.41</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>9601576.18</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>8364421.16</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>1237155.01</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>4.8088</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>971.03</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>95.48999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-25 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1284,6 +1284,37 @@
         <v>95.48999999999999</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>9645997.050000001</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>8365373.76</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>1280623.28</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>4.8651</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>975.53</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>81.63</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>95.42</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-26 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1315,6 +1315,37 @@
         <v>95.42</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>9893</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>9505509.550000001</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>8195018.89</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>1310490.65</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>4.8661</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>960.83</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>80.73</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>95.26000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-27 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1346,6 +1346,37 @@
         <v>95.26000000000001</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>9911</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>9498573.119999999</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>8196600.87</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>1301972.25</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>4.8526</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>958.39</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>80.83</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>95.20999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-28 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1377,6 +1377,37 @@
         <v>95.20999999999999</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>9925</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>9488256.4</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>8198037.32</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>1290219.08</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>4.8502</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>956</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>80.91</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>95.18000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-29 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1408,6 +1408,37 @@
         <v>95.18000000000001</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>9846</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>9561988.439999999</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>8271707.56</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>1290280.89</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>4.7794</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>971.15</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>82.66</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>95.87</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-30 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1439,6 +1439,37 @@
         <v>95.87</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>9853</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>9618208.140000001</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>8272314.57</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>1345893.57</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>4.7932</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>976.17</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>82.17</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>95.88</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-07-31 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1470,6 +1470,37 @@
         <v>95.88</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>9853</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>9678783.6</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>8303210.42</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>1375573.19</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>4.7925</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>982.3200000000001</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>81.65000000000001</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>95.84999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-01 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1501,6 +1501,37 @@
         <v>95.84999999999999</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>9860</v>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>9564077.390000001</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>8298561.31</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>1265516.08</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>4.7903</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>969.99</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>82.61</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>95.84999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-02 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1532,6 +1532,37 @@
         <v>95.84999999999999</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>9856</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>9466838.85</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>8200198.58</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>1266640.27</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>4.7858</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>960.52</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>95.79000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-03 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1563,6 +1563,37 @@
         <v>95.79000000000001</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>9858</v>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>9455564.16</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>8198099.26</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>1257464.9</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>4.7925</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>959.1799999999999</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>82.48999999999999</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>95.83</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-04 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1594,6 +1594,37 @@
         <v>95.83</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>9848</v>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>9439797.76</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>8188011.71</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>1251786.05</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>4.7932</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>958.55</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>82.63</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>95.84</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-05 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1625,6 +1625,37 @@
         <v>95.84</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>9858</v>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>9438663.65</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>8186673.25</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>1251990.4</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>4.7809</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>957.46</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>82.62</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>95.84</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-06 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1656,6 +1656,37 @@
         <v>95.84</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>9859</v>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>10636565.11</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>9387690.949999999</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>1248874.16</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>4.777</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>1078.87</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>82.14</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>96.27</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-07 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1687,6 +1687,37 @@
         <v>96.27</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>9862</v>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>10635710.45</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>9386562.390000001</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>1249148.06</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>4.7809</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>1078.45</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>96.27</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-08 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1718,6 +1718,37 @@
         <v>96.27</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>9863</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>10633038.84</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>9388953.6</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>1244085.24</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>4.7794</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>1078.07</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>82.17</v>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>96.29000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-09 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1749,6 +1749,37 @@
         <v>96.29000000000001</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>9850</v>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>10614898.28</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>9392617.84</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>1222280.45</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>4.7719</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>1077.65</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>82.31</v>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>96.38</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-10 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1780,6 +1780,37 @@
         <v>96.38</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>9765</v>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>10603890.86</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>9392028.529999999</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>1211862.33</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>4.621</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>1085.91</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>82.39</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>96.38</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-11 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1811,6 +1811,37 @@
         <v>96.38</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>9760</v>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>10594048.97</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>9380630.98</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>1213417.98</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>4.621</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>1085.46</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>82.47</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>96.40000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-12 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1842,6 +1842,37 @@
         <v>96.40000000000001</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>9788</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>10608958.87</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>9384419.960000001</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>1224538.91</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>4.6095</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>1083.87</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>82.34</v>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>96.38</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-13 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1873,6 +1873,37 @@
         <v>96.38</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>9786</v>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>10569136.81</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>9382675.720000001</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>1186461.1</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>4.621</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>1080.03</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>82.65000000000001</v>
+      </c>
+      <c r="I47" s="5" t="n">
+        <v>96.41</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-15 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1904,6 +1904,37 @@
         <v>96.41</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>9722</v>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>10452262.9</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>9292070.529999999</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>1160192.37</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>4.4932</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>1075.11</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>83.58</v>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>96.39</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-16 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1935,6 +1935,37 @@
         <v>96.39</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>9711</v>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>10401024.1</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>9285073.880000001</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>1115950.23</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>4.4459</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>1071.06</v>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="I49" s="5" t="n">
+        <v>96.45999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-17 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1966,6 +1966,37 @@
         <v>96.45999999999999</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>9703</v>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>10606972.11</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>9204274.060000001</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>1402698.05</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>4.4435</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>1093.16</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>81.42</v>
+      </c>
+      <c r="I50" s="5" t="n">
+        <v>96.51000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-18 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1997,6 +1997,37 @@
         <v>96.51000000000001</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>9698</v>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>10643189.32</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>9150799.1</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>1492390.22</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>4.4627</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>1097.46</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>81.13</v>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>96.56</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-19 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2028,6 +2028,37 @@
         <v>96.56</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>9692</v>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>10616549.26</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>9140807.15</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>1475742.11</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>4.4529</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>1095.39</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>81.29000000000001</v>
+      </c>
+      <c r="I52" s="5" t="n">
+        <v>96.52</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-20 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2059,6 +2059,37 @@
         <v>96.52</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>9479</v>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>10658732.76</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>9143271.300000001</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>1515461.47</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>4.1871</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>1124.46</v>
+      </c>
+      <c r="H53" s="5" t="n">
+        <v>80.97</v>
+      </c>
+      <c r="I53" s="5" t="n">
+        <v>96.59</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-21 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2090,6 +2090,37 @@
         <v>96.59</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>9433</v>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>10610198.5</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>9145748.109999999</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>1464450.38</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>4.1489</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>1124.8</v>
+      </c>
+      <c r="H54" s="5" t="n">
+        <v>81.34</v>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>96.51000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-22 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2121,6 +2121,37 @@
         <v>96.51000000000001</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>9408</v>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>10666409.5</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>9159442.289999999</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>1506967.21</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>4.1152</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>1133.76</v>
+      </c>
+      <c r="H55" s="5" t="n">
+        <v>80.91</v>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>96.56</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-23 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2152,6 +2152,37 @@
         <v>96.56</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>9167</v>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>10571347.44</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>9141094.9</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>1430252.54</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>3.9748</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>1153.2</v>
+      </c>
+      <c r="H56" s="5" t="n">
+        <v>81.64</v>
+      </c>
+      <c r="I56" s="5" t="n">
+        <v>96.54000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-24 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2183,6 +2183,37 @@
         <v>96.54000000000001</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>9046</v>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>10563050.72</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>9141326.199999999</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>1421724.52</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>3.8462</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>1167.7</v>
+      </c>
+      <c r="H57" s="5" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="I57" s="5" t="n">
+        <v>96.54000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-25 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2214,6 +2214,37 @@
         <v>96.54000000000001</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>9060</v>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>10586588.07</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>9142370.460000001</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>1444217.61</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>3.8283</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>1168.5</v>
+      </c>
+      <c r="H58" s="5" t="n">
+        <v>81.52</v>
+      </c>
+      <c r="I58" s="5" t="n">
+        <v>96.52</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-26 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2245,6 +2245,37 @@
         <v>96.52</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n">
+        <v>9062</v>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>10575435</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>9141969.49</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>1433465.51</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>3.8206</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>1167.01</v>
+      </c>
+      <c r="H59" s="5" t="n">
+        <v>81.61</v>
+      </c>
+      <c r="I59" s="5" t="n">
+        <v>96.52</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-27 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2276,6 +2276,37 @@
         <v>96.52</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="n">
+        <v>9068</v>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>10588271.52</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>9142119.279999999</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>1446152.24</v>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>3.8625</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>1167.65</v>
+      </c>
+      <c r="H60" s="5" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="I60" s="5" t="n">
+        <v>96.5</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-28 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2307,6 +2307,37 @@
         <v>96.5</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="n">
+        <v>9063</v>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>10597597.17</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>9136640.119999999</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>1460957.06</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>3.8631</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>1169.33</v>
+      </c>
+      <c r="H61" s="5" t="n">
+        <v>81.43000000000001</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>96.5</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-29 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2338,6 +2338,37 @@
         <v>96.5</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="n">
+        <v>9062</v>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>10585012.89</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>9135789.859999999</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>1449223.03</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>3.8462</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>1168.07</v>
+      </c>
+      <c r="H62" s="5" t="n">
+        <v>81.53</v>
+      </c>
+      <c r="I62" s="5" t="n">
+        <v>96.5</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-30 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2369,6 +2369,37 @@
         <v>96.5</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="n">
+        <v>9045</v>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>10551674.74</v>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>9135394.460000001</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>1416280.29</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>3.8283</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>1166.58</v>
+      </c>
+      <c r="H63" s="5" t="n">
+        <v>81.78</v>
+      </c>
+      <c r="I63" s="5" t="n">
+        <v>96.51000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-08-31 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2400,6 +2400,37 @@
         <v>96.51000000000001</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="n">
+        <v>9015</v>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>10358124.57</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>9134263.32</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>1223861.25</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>3.8683</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>1148.99</v>
+      </c>
+      <c r="H64" s="5" t="n">
+        <v>83.31</v>
+      </c>
+      <c r="I64" s="5" t="n">
+        <v>96.41</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-01 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2431,6 +2431,37 @@
         <v>96.41</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="n">
+        <v>8989</v>
+      </c>
+      <c r="C65" s="3" t="n">
+        <v>10374125.13</v>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>9135300.84</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>1238824.29</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>3.8223</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>1154.09</v>
+      </c>
+      <c r="H65" s="5" t="n">
+        <v>83.18000000000001</v>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>96.62</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-02 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2462,6 +2462,37 @@
         <v>96.62</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="n">
+        <v>8984</v>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>10389467.87</v>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>9135810.1</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>1253657.77</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>3.8076</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>1156.44</v>
+      </c>
+      <c r="H66" s="5" t="n">
+        <v>83.06</v>
+      </c>
+      <c r="I66" s="5" t="n">
+        <v>96.59</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-03 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2493,6 +2493,37 @@
         <v>96.59</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="n">
+        <v>8984</v>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>10372741.83</v>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>9127726.720000001</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>1245015.11</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>1154.58</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="I67" s="5" t="n">
+        <v>96.67</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-04 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2524,6 +2524,37 @@
         <v>96.67</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="n">
+        <v>8985</v>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>10393875.59</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>9133050.9</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>1260824.69</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>3.8165</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>1156.8</v>
+      </c>
+      <c r="H68" s="5" t="n">
+        <v>83.02</v>
+      </c>
+      <c r="I68" s="5" t="n">
+        <v>96.69</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-05 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2555,6 +2555,37 @@
         <v>96.69</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="n">
+        <v>8988</v>
+      </c>
+      <c r="C69" s="3" t="n">
+        <v>10363283.18</v>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>9135133.890000001</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>1228149.29</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>3.8185</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>1153.01</v>
+      </c>
+      <c r="H69" s="5" t="n">
+        <v>83.27</v>
+      </c>
+      <c r="I69" s="5" t="n">
+        <v>96.72</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-06 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2586,6 +2586,37 @@
         <v>96.72</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="n">
+        <v>8989</v>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>10365148.89</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>9137631.130000001</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>1227517.76</v>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>3.8218</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>1153.09</v>
+      </c>
+      <c r="H70" s="5" t="n">
+        <v>83.25</v>
+      </c>
+      <c r="I70" s="5" t="n">
+        <v>96.7</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-07 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2617,6 +2617,37 @@
         <v>96.7</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="n">
+        <v>8990</v>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>10368107.91</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>9139990.470000001</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>1228117.43</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>3.8185</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>1153.29</v>
+      </c>
+      <c r="H71" s="5" t="n">
+        <v>83.22</v>
+      </c>
+      <c r="I71" s="5" t="n">
+        <v>96.72</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-08 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2648,6 +2648,37 @@
         <v>96.72</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="n">
+        <v>9007</v>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>10366896.35</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>9142404.960000001</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>1224491.39</v>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>3.8426</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>1150.98</v>
+      </c>
+      <c r="H72" s="5" t="n">
+        <v>83.23</v>
+      </c>
+      <c r="I72" s="5" t="n">
+        <v>96.73999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-09 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2679,6 +2679,37 @@
         <v>96.73999999999999</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="n">
+        <v>9009</v>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>10365188.84</v>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>9142741.49</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>1222447.35</v>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>3.8705</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>1150.54</v>
+      </c>
+      <c r="H73" s="5" t="n">
+        <v>83.23999999999999</v>
+      </c>
+      <c r="I73" s="5" t="n">
+        <v>96.73999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-10 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2710,6 +2710,37 @@
         <v>96.73999999999999</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="n">
+        <v>9019</v>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>10377635.67</v>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>9154562.890000001</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>1223072.77</v>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>3.8631</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>1150.64</v>
+      </c>
+      <c r="H74" s="5" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="I74" s="5" t="n">
+        <v>96.70999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-11 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2741,6 +2741,37 @@
         <v>96.70999999999999</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="n">
+        <v>9009</v>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>10358837.65</v>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>9142539.91</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>1216297.74</v>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>3.8704</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>1149.83</v>
+      </c>
+      <c r="H75" s="5" t="n">
+        <v>83.29000000000001</v>
+      </c>
+      <c r="I75" s="5" t="n">
+        <v>96.72</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-12 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2772,6 +2772,37 @@
         <v>96.72</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="n">
+        <v>9019</v>
+      </c>
+      <c r="C76" s="3" t="n">
+        <v>10357594.81</v>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>9139074.380000001</v>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>1218520.43</v>
+      </c>
+      <c r="F76" s="4" t="n">
+        <v>3.8777</v>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>1148.42</v>
+      </c>
+      <c r="H76" s="5" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="I76" s="5" t="n">
+        <v>96.73</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-13 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2803,6 +2803,37 @@
         <v>96.73</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="n">
+        <v>9026</v>
+      </c>
+      <c r="C77" s="3" t="n">
+        <v>10357882.33</v>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>9138785.52</v>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>1219096.8</v>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>3.8704</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>1147.56</v>
+      </c>
+      <c r="H77" s="5" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>96.73</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>